<commit_message>
fix: handle floatingpoints errors coming from excel
</commit_message>
<xml_diff>
--- a/examples/test/testFiles/TwoRowsNoErrors.xlsx
+++ b/examples/test/testFiles/TwoRowsNoErrors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianzeis/DEV/ui5-cc-excelUpload/examples/test/testFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianzeis/DEV/ui5-cc-spreadsheetimporter/examples/test/testFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F2FC3F6-0198-0042-8CAE-C4B968E0CFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CA5A1B-93B1-5742-B7D1-E9E15F758C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="30240" windowHeight="17660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,7 +127,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -583,7 +583,7 @@
         <v>12</v>
       </c>
       <c r="J3">
-        <v>14.3</v>
+        <v>1.2199999999999999E-2</v>
       </c>
       <c r="K3">
         <v>4</v>

</xml_diff>

<commit_message>
fix: handle floatingpoints errors coming from excel (#789)
</commit_message>
<xml_diff>
--- a/examples/test/testFiles/TwoRowsNoErrors.xlsx
+++ b/examples/test/testFiles/TwoRowsNoErrors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianzeis/DEV/ui5-cc-excelUpload/examples/test/testFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianzeis/DEV/ui5-cc-spreadsheetimporter/examples/test/testFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F2FC3F6-0198-0042-8CAE-C4B968E0CFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CA5A1B-93B1-5742-B7D1-E9E15F758C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="30240" windowHeight="17660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,7 +127,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -583,7 +583,7 @@
         <v>12</v>
       </c>
       <c r="J3">
-        <v>14.3</v>
+        <v>1.2199999999999999E-2</v>
       </c>
       <c r="K3">
         <v>4</v>

</xml_diff>